<commit_message>
feat: Add reusable common UI widgets
</commit_message>
<xml_diff>
--- a/PRICE LIST.xlsx
+++ b/PRICE LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PROJECT\LF_KITCHEN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28ADE9E3-F408-4E55-A3C9-9855EB1AC30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BC9C4A-4201-4812-949A-3BEF6D30A682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DB740CC4-E712-4A4C-BF70-FD0CED442F24}"/>
   </bookViews>
@@ -296,7 +296,7 @@
   <numFmts count="1">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -313,20 +313,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -360,16 +346,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -694,7 +674,7 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C2" s="1">
@@ -718,7 +698,7 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>79</v>
       </c>
       <c r="C3" s="1">
@@ -741,7 +721,7 @@
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C4" s="1">
@@ -764,7 +744,7 @@
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C5" s="1">
@@ -787,7 +767,7 @@
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C6" s="1">
@@ -810,7 +790,7 @@
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C7" s="1">
@@ -834,7 +814,7 @@
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C8" s="1">
@@ -858,7 +838,7 @@
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C9" s="1">
@@ -882,7 +862,7 @@
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C10" s="1">
@@ -906,7 +886,7 @@
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C11" s="1">
@@ -930,7 +910,7 @@
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C12" s="1">
@@ -954,7 +934,7 @@
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C13" s="1">
@@ -978,7 +958,7 @@
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C14" s="1">
@@ -1002,7 +982,7 @@
       <c r="A15" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C15" s="1">
@@ -1026,7 +1006,7 @@
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C16" s="1">
@@ -1050,7 +1030,7 @@
       <c r="A17" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C17" s="1">
@@ -1074,7 +1054,7 @@
       <c r="A18" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C18" s="1">
@@ -1098,7 +1078,7 @@
       <c r="A19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C19" s="1">
@@ -1122,7 +1102,7 @@
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C20" s="1">
@@ -1146,7 +1126,7 @@
       <c r="A21" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C21" s="1">
@@ -1170,7 +1150,7 @@
       <c r="A22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C22" s="1">
@@ -1194,7 +1174,7 @@
       <c r="A23" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C23" s="1">
@@ -1217,7 +1197,7 @@
       <c r="A24" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C24" s="1">
@@ -1240,7 +1220,7 @@
       <c r="A25" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C25" s="1">
@@ -1263,7 +1243,7 @@
       <c r="A26" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C26" s="1">
@@ -1283,7 +1263,7 @@
       <c r="A27" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C27" s="1">
@@ -1303,7 +1283,7 @@
       <c r="A28" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C28" s="1">
@@ -1323,7 +1303,7 @@
       <c r="A29" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C29" s="1">
@@ -1346,7 +1326,7 @@
       <c r="A30" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C30" s="1">
@@ -1369,7 +1349,7 @@
       <c r="A31" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C31" s="1">
@@ -1392,7 +1372,7 @@
       <c r="A32" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C32" s="1">
@@ -1415,10 +1395,12 @@
       <c r="A33" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C33" s="3"/>
+      <c r="C33" s="1">
+        <v>55000</v>
+      </c>
       <c r="D33" s="1">
         <v>55000</v>
       </c>
@@ -1436,10 +1418,12 @@
       <c r="A34" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B34" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C34" s="3"/>
+      <c r="B34" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C34" s="1">
+        <v>95000</v>
+      </c>
       <c r="D34" s="1">
         <v>95000</v>
       </c>
@@ -1457,10 +1441,12 @@
       <c r="A35" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C35" s="3"/>
+      <c r="C35" s="1">
+        <v>50000</v>
+      </c>
       <c r="D35" s="1">
         <v>50000</v>
       </c>
@@ -1478,10 +1464,12 @@
       <c r="A36" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C36" s="3"/>
+      <c r="B36" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="1">
+        <v>80000</v>
+      </c>
       <c r="D36" s="1">
         <v>80000</v>
       </c>
@@ -1499,10 +1487,12 @@
       <c r="A37" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C37" s="3"/>
+      <c r="C37" s="1">
+        <v>50000</v>
+      </c>
       <c r="D37" s="1">
         <v>50000</v>
       </c>
@@ -1520,10 +1510,12 @@
       <c r="A38" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C38" s="3"/>
+      <c r="B38" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" s="1">
+        <v>80000</v>
+      </c>
       <c r="D38" s="1">
         <v>80000</v>
       </c>
@@ -1541,10 +1533,12 @@
       <c r="A39" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C39" s="3"/>
+      <c r="C39" s="1">
+        <v>65000</v>
+      </c>
       <c r="D39" s="1">
         <v>65000</v>
       </c>
@@ -1562,10 +1556,12 @@
       <c r="A40" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C40" s="3"/>
+      <c r="B40" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C40" s="1">
+        <v>110000</v>
+      </c>
       <c r="D40" s="1">
         <v>110000</v>
       </c>
@@ -1583,10 +1579,12 @@
       <c r="A41" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C41" s="3"/>
+      <c r="C41" s="1">
+        <v>50000</v>
+      </c>
       <c r="D41" s="1">
         <v>50000</v>
       </c>
@@ -1604,10 +1602,12 @@
       <c r="A42" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C42" s="3"/>
+      <c r="B42" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="1">
+        <v>85000</v>
+      </c>
       <c r="D42" s="1">
         <v>85000</v>
       </c>
@@ -1625,10 +1625,12 @@
       <c r="A43" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C43" s="3"/>
+      <c r="C43" s="1">
+        <v>60000</v>
+      </c>
       <c r="D43" s="1">
         <v>60000</v>
       </c>
@@ -1646,10 +1648,12 @@
       <c r="A44" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C44" s="3"/>
+      <c r="B44" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="1">
+        <v>105000</v>
+      </c>
       <c r="D44" s="1">
         <v>105000</v>
       </c>
@@ -1667,10 +1671,12 @@
       <c r="A45" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C45" s="3"/>
+      <c r="C45" s="1">
+        <v>50000</v>
+      </c>
       <c r="D45" s="1">
         <v>50000</v>
       </c>
@@ -1688,10 +1694,12 @@
       <c r="A46" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B46" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C46" s="3"/>
+      <c r="B46" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C46" s="1">
+        <v>80000</v>
+      </c>
       <c r="D46" s="1">
         <v>80000</v>
       </c>
@@ -1709,10 +1717,12 @@
       <c r="A47" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C47" s="3"/>
+      <c r="C47" s="1">
+        <v>50000</v>
+      </c>
       <c r="D47" s="1">
         <v>50000</v>
       </c>
@@ -1730,10 +1740,12 @@
       <c r="A48" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B48" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C48" s="3"/>
+      <c r="B48" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C48" s="1">
+        <v>90000</v>
+      </c>
       <c r="D48" s="1">
         <v>90000</v>
       </c>
@@ -1751,10 +1763,12 @@
       <c r="A49" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C49" s="3"/>
+      <c r="C49" s="1">
+        <v>50000</v>
+      </c>
       <c r="D49" s="1">
         <v>50000</v>
       </c>
@@ -1772,10 +1786,12 @@
       <c r="A50" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C50" s="3"/>
+      <c r="B50" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C50" s="1">
+        <v>80000</v>
+      </c>
       <c r="D50" s="1">
         <v>80000</v>
       </c>
@@ -1793,10 +1809,12 @@
       <c r="A51" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C51" s="3"/>
+      <c r="C51" s="1">
+        <v>50000</v>
+      </c>
       <c r="D51" s="1">
         <v>50000</v>
       </c>
@@ -1814,10 +1832,12 @@
       <c r="A52" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B52" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C52" s="3"/>
+      <c r="B52" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C52" s="1">
+        <v>80000</v>
+      </c>
       <c r="D52" s="1">
         <v>80000</v>
       </c>
@@ -1835,10 +1855,12 @@
       <c r="A53" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C53" s="3"/>
+      <c r="B53" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C53" s="1">
+        <v>3500</v>
+      </c>
       <c r="D53" s="1">
         <v>3500</v>
       </c>
@@ -1856,8 +1878,11 @@
       <c r="A54" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>78</v>
+      <c r="B54" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C54" s="1">
+        <v>13000</v>
       </c>
       <c r="D54" s="1">
         <v>13000</v>
@@ -1876,10 +1901,12 @@
       <c r="A55" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C55" s="3"/>
+      <c r="B55" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C55" s="1">
+        <v>55000</v>
+      </c>
       <c r="D55" s="1">
         <v>55000</v>
       </c>
@@ -1897,10 +1924,12 @@
       <c r="A56" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C56" s="3"/>
+      <c r="B56" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C56" s="1">
+        <v>45000</v>
+      </c>
       <c r="D56" s="1">
         <v>45000</v>
       </c>
@@ -1918,10 +1947,12 @@
       <c r="A57" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B57" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C57" s="3"/>
+      <c r="B57" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C57" s="1">
+        <v>50000</v>
+      </c>
       <c r="D57" s="1">
         <v>50000</v>
       </c>
@@ -1939,10 +1970,12 @@
       <c r="A58" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B58" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C58" s="3"/>
+      <c r="B58" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C58" s="1">
+        <v>50000</v>
+      </c>
       <c r="D58" s="1">
         <v>50000</v>
       </c>
@@ -1960,10 +1993,12 @@
       <c r="A59" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C59" s="3"/>
+      <c r="B59" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C59" s="1">
+        <v>50000</v>
+      </c>
       <c r="D59" s="1">
         <v>50000</v>
       </c>
@@ -1981,10 +2016,12 @@
       <c r="A60" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C60" s="3"/>
+      <c r="B60" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C60" s="1">
+        <v>55000</v>
+      </c>
       <c r="D60" s="1">
         <v>55000</v>
       </c>
@@ -2002,10 +2039,12 @@
       <c r="A61" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C61" s="3"/>
+      <c r="B61" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C61" s="1">
+        <v>60000</v>
+      </c>
       <c r="D61" s="1">
         <v>60000</v>
       </c>
@@ -2023,10 +2062,12 @@
       <c r="A62" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C62" s="3"/>
+      <c r="B62" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C62" s="1">
+        <v>25000</v>
+      </c>
       <c r="D62" s="1">
         <v>25000</v>
       </c>
@@ -2044,10 +2085,12 @@
       <c r="A63" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C63" s="3"/>
+      <c r="B63" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C63" s="1">
+        <v>25000</v>
+      </c>
       <c r="D63" s="1">
         <v>25000</v>
       </c>
@@ -2065,10 +2108,12 @@
       <c r="A64" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C64" s="3"/>
+      <c r="B64" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C64" s="1">
+        <v>25000</v>
+      </c>
       <c r="D64" s="1">
         <v>25000</v>
       </c>
@@ -2086,10 +2131,12 @@
       <c r="A65" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B65" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C65" s="3"/>
+      <c r="B65" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C65" s="1">
+        <v>30000</v>
+      </c>
       <c r="D65" s="1">
         <v>30000</v>
       </c>
@@ -2107,10 +2154,12 @@
       <c r="A66" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B66" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C66" s="3"/>
+      <c r="B66" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C66" s="1">
+        <v>60000</v>
+      </c>
       <c r="D66" s="1">
         <v>60000</v>
       </c>
@@ -2128,10 +2177,12 @@
       <c r="A67" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B67" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C67" s="3"/>
+      <c r="B67" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C67" s="1">
+        <v>65000</v>
+      </c>
       <c r="D67" s="1">
         <v>65000</v>
       </c>
@@ -2149,10 +2200,12 @@
       <c r="A68" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C68" s="3"/>
+      <c r="B68" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C68" s="1">
+        <v>65000</v>
+      </c>
       <c r="D68" s="1">
         <v>65000</v>
       </c>
@@ -2170,10 +2223,12 @@
       <c r="A69" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B69" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C69" s="3"/>
+      <c r="B69" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C69" s="1">
+        <v>65000</v>
+      </c>
       <c r="D69" s="1">
         <v>65000</v>
       </c>
@@ -2191,10 +2246,12 @@
       <c r="A70" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B70" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C70" s="3"/>
+      <c r="B70" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C70" s="1">
+        <v>65000</v>
+      </c>
       <c r="D70" s="1">
         <v>65000</v>
       </c>
@@ -2212,10 +2269,12 @@
       <c r="A71" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B71" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C71" s="3"/>
+      <c r="B71" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C71" s="1">
+        <v>70000</v>
+      </c>
       <c r="D71" s="1">
         <v>70000</v>
       </c>
@@ -2233,10 +2292,12 @@
       <c r="A72" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B72" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C72" s="3"/>
+      <c r="B72" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C72" s="1">
+        <v>85000</v>
+      </c>
       <c r="D72" s="1">
         <v>85000</v>
       </c>
@@ -2254,10 +2315,12 @@
       <c r="A73" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B73" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C73" s="3"/>
+      <c r="B73" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C73" s="1">
+        <v>150000</v>
+      </c>
       <c r="D73" s="1">
         <v>150000</v>
       </c>
@@ -2275,10 +2338,12 @@
       <c r="A74" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B74" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C74" s="4"/>
+      <c r="B74" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C74" s="1">
+        <v>50000</v>
+      </c>
       <c r="D74" s="1">
         <v>50000</v>
       </c>
@@ -2296,10 +2361,12 @@
       <c r="A75" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B75" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C75" s="3"/>
+      <c r="B75" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C75" s="1">
+        <v>70000</v>
+      </c>
       <c r="D75" s="1">
         <v>70000</v>
       </c>
@@ -2317,10 +2384,12 @@
       <c r="A76" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B76" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C76" s="3"/>
+      <c r="B76" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C76" s="1">
+        <v>70000</v>
+      </c>
       <c r="D76" s="1">
         <v>70000</v>
       </c>

</xml_diff>

<commit_message>
feat: Add Excel import/export and database reset script
</commit_message>
<xml_diff>
--- a/PRICE LIST.xlsx
+++ b/PRICE LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PROJECT\LF_KITCHEN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BC9C4A-4201-4812-949A-3BEF6D30A682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DD65668-E17E-4BCF-86C8-88AD1A9A11D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DB740CC4-E712-4A4C-BF70-FD0CED442F24}"/>
   </bookViews>
@@ -277,9 +277,6 @@
     <t>SMALL</t>
   </si>
   <si>
-    <t>BIG</t>
-  </si>
-  <si>
     <t>JENIS</t>
   </si>
   <si>
@@ -287,6 +284,9 @@
   </si>
   <si>
     <t>MANIS</t>
+  </si>
+  <si>
+    <t>LARGE</t>
   </si>
 </sst>
 </file>
@@ -667,7 +667,7 @@
         <v>64</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -691,7 +691,7 @@
         <v>65</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -714,7 +714,7 @@
         <v>65</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -722,7 +722,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C4" s="1">
         <v>5000</v>
@@ -737,7 +737,7 @@
         <v>65</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -760,7 +760,7 @@
         <v>65</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -783,7 +783,7 @@
         <v>65</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -794,7 +794,7 @@
         <v>78</v>
       </c>
       <c r="C7" s="1">
-        <f t="shared" ref="C7:C22" si="0">D7+500</f>
+        <f t="shared" ref="C7:C23" si="0">D7+500</f>
         <v>3500</v>
       </c>
       <c r="D7" s="1">
@@ -807,7 +807,7 @@
         <v>65</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -831,7 +831,7 @@
         <v>65</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -855,7 +855,7 @@
         <v>65</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -879,7 +879,7 @@
         <v>65</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -903,7 +903,7 @@
         <v>65</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -927,7 +927,7 @@
         <v>65</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -951,7 +951,7 @@
         <v>65</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -975,71 +975,70 @@
         <v>65</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="1">
+        <v>3000</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2500</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C15" s="1">
+      <c r="B16" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="1">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D16" s="1">
         <v>3500</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="E16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="1">
+      <c r="B17" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="1">
         <f t="shared" si="0"/>
         <v>3500</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D17" s="1">
         <v>3000</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="1">
-        <f t="shared" si="0"/>
-        <v>4000</v>
-      </c>
-      <c r="D17" s="1">
-        <v>3500</v>
-      </c>
       <c r="E17" s="1" t="s">
         <v>61</v>
       </c>
@@ -1047,12 +1046,12 @@
         <v>65</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>78</v>
@@ -1071,12 +1070,12 @@
         <v>65</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>78</v>
@@ -1095,12 +1094,12 @@
         <v>65</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>78</v>
@@ -1119,12 +1118,12 @@
         <v>65</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>78</v>
@@ -1143,22 +1142,22 @@
         <v>65</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C22" s="1">
         <f t="shared" si="0"/>
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="D22" s="1">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>61</v>
@@ -1167,17 +1166,18 @@
         <v>65</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C23" s="1">
+        <f t="shared" si="0"/>
         <v>3000</v>
       </c>
       <c r="D23" s="1">
@@ -1190,12 +1190,12 @@
         <v>65</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>78</v>
@@ -1213,12 +1213,12 @@
         <v>65</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>78</v>
@@ -1319,7 +1319,7 @@
         <v>65</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1342,7 +1342,7 @@
         <v>65</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1365,7 +1365,7 @@
         <v>65</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1388,7 +1388,7 @@
         <v>65</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1411,7 +1411,7 @@
         <v>69</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1434,7 +1434,7 @@
         <v>69</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1457,7 +1457,7 @@
         <v>69</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -1480,7 +1480,7 @@
         <v>69</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -1503,7 +1503,7 @@
         <v>69</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -1526,7 +1526,7 @@
         <v>69</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -1549,7 +1549,7 @@
         <v>69</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -1572,7 +1572,7 @@
         <v>69</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -1595,7 +1595,7 @@
         <v>69</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -1618,7 +1618,7 @@
         <v>69</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -1641,7 +1641,7 @@
         <v>69</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -1664,7 +1664,7 @@
         <v>69</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -1687,7 +1687,7 @@
         <v>69</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -1710,7 +1710,7 @@
         <v>69</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -1733,7 +1733,7 @@
         <v>69</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -1756,7 +1756,7 @@
         <v>69</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -1779,7 +1779,7 @@
         <v>69</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
@@ -1802,7 +1802,7 @@
         <v>69</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -1825,7 +1825,7 @@
         <v>69</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -1848,7 +1848,7 @@
         <v>69</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -1871,7 +1871,7 @@
         <v>65</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -1894,7 +1894,7 @@
         <v>70</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -1917,7 +1917,7 @@
         <v>71</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
@@ -1940,7 +1940,7 @@
         <v>71</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -1963,7 +1963,7 @@
         <v>71</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
@@ -1986,7 +1986,7 @@
         <v>71</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -2009,7 +2009,7 @@
         <v>71</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
@@ -2032,7 +2032,7 @@
         <v>71</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
@@ -2055,7 +2055,7 @@
         <v>71</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
@@ -2078,7 +2078,7 @@
         <v>71</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
@@ -2101,7 +2101,7 @@
         <v>71</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
@@ -2124,7 +2124,7 @@
         <v>71</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
@@ -2147,7 +2147,7 @@
         <v>71</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
@@ -2170,7 +2170,7 @@
         <v>71</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
@@ -2193,7 +2193,7 @@
         <v>71</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
@@ -2216,7 +2216,7 @@
         <v>71</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
@@ -2239,7 +2239,7 @@
         <v>71</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
@@ -2262,7 +2262,7 @@
         <v>71</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
@@ -2285,7 +2285,7 @@
         <v>71</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
@@ -2308,7 +2308,7 @@
         <v>71</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
@@ -2331,7 +2331,7 @@
         <v>71</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
@@ -2354,7 +2354,7 @@
         <v>71</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
@@ -2377,7 +2377,7 @@
         <v>71</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
@@ -2400,7 +2400,7 @@
         <v>71</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>